<commit_message>
GBDS AUG 2026 | berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS AUGUST FILES 2026/CSR MONTH OF AUGUST 2026.xlsx
+++ b/GBDS AUGUST FILES 2026/CSR MONTH OF AUGUST 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS AUGUST FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363B052C-31CF-4EF8-84ED-50F82723D379}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2D16E9-3AA3-48EC-963E-AA75FD268CCC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="12" activeTab="14" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="18" activeTab="19" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | AUGUST" sheetId="902" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="08-05 R2" sheetId="1865" r:id="rId16"/>
     <sheet name="08-05 R3 NO TRIP" sheetId="1866" r:id="rId17"/>
     <sheet name="(6)" sheetId="1867" r:id="rId18"/>
-    <sheet name="08-06 R1" sheetId="1868" r:id="rId19"/>
+    <sheet name="08-06 R1 NO TRIP" sheetId="1868" r:id="rId19"/>
     <sheet name="08-06 R2" sheetId="1869" r:id="rId20"/>
     <sheet name="08-06 R3" sheetId="1870" r:id="rId21"/>
     <sheet name="(7)" sheetId="1871" r:id="rId22"/>
@@ -68,7 +68,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="14">'08-05 R1'!$A$1:$Z$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="15">'08-05 R2'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="16">'08-05 R3 NO TRIP'!$A$1:$V$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="18">'08-06 R1'!$A$1:$Z$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="18">'08-06 R1 NO TRIP'!$A$1:$Z$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="19">'08-06 R2'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="20">'08-06 R3'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="22">'08-07 R1'!$A$1:$Z$43</definedName>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2851" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2860" uniqueCount="101">
   <si>
     <t>CHECKER STOCK REPORT</t>
   </si>
@@ -382,6 +382,24 @@
   </si>
   <si>
     <t>10/10B</t>
+  </si>
+  <si>
+    <t>11/5B</t>
+  </si>
+  <si>
+    <t>5B</t>
+  </si>
+  <si>
+    <t>11/10B</t>
+  </si>
+  <si>
+    <t>1/12B</t>
+  </si>
+  <si>
+    <t>11/12B</t>
+  </si>
+  <si>
+    <t>5/3B</t>
   </si>
 </sst>
 </file>
@@ -1002,7 +1020,7 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1263,6 +1281,9 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2824,47 +2845,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -3096,12 +3117,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -4355,47 +4376,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -4627,12 +4648,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -4668,17 +4689,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -5974,47 +5995,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -6270,12 +6291,12 @@
       <c r="Q42" s="43">
         <v>5</v>
       </c>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -6311,23 +6332,23 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>11+20+2+431</f>
         <v>464</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95">
+      <c r="C45" s="96">
         <f>4</f>
         <v>4</v>
       </c>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7617,47 +7638,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -7929,12 +7950,12 @@
       <c r="Q42" s="43">
         <v>2</v>
       </c>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -7970,23 +7991,23 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>17+2+4+55+4+548</f>
         <v>630</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95">
+      <c r="C45" s="96">
         <f>5</f>
         <v>5</v>
       </c>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9207,47 +9228,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -9479,12 +9500,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -10792,47 +10813,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -11108,12 +11129,12 @@
       <c r="Q42" s="43">
         <v>1</v>
       </c>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -11149,20 +11170,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>8+113+15+236</f>
         <v>372</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -12476,47 +12497,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -12792,12 +12813,12 @@
         <v>6</v>
       </c>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -12833,22 +12854,22 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>2+10+1+1+1+21+1+322+1</f>
         <v>360</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95">
+      <c r="C45" s="96">
         <v>10</v>
       </c>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -14072,47 +14093,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -14344,12 +14365,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -14385,17 +14406,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -15616,47 +15637,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -15888,12 +15909,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -17147,47 +17168,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -17419,12 +17440,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -17460,17 +17481,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -18691,47 +18712,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -18963,12 +18984,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -19356,12 +19377,18 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="77"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="13">
+        <v>1</v>
+      </c>
+      <c r="D8" s="14">
+        <v>1</v>
+      </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14">
+        <v>13</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -19376,7 +19403,9 @@
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>2</v>
+      </c>
       <c r="X8" s="59"/>
       <c r="Y8" s="15"/>
     </row>
@@ -19544,12 +19573,18 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
+      <c r="D15" s="23">
+        <v>1</v>
+      </c>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>98</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -19564,7 +19599,9 @@
       <c r="T15" s="23"/>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>2</v>
+      </c>
       <c r="X15" s="61"/>
       <c r="Y15" s="24"/>
     </row>
@@ -19572,12 +19609,18 @@
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
+      <c r="C16" s="57">
+        <v>0</v>
+      </c>
+      <c r="D16" s="58">
+        <v>0</v>
+      </c>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>99</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -19592,7 +19635,9 @@
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
+      <c r="W16" s="56">
+        <v>0</v>
+      </c>
       <c r="X16" s="62"/>
       <c r="Y16" s="29"/>
     </row>
@@ -19958,23 +20003,37 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="78"/>
+      <c r="F24" s="14">
+        <v>3</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>29</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>69</v>
+      </c>
+      <c r="L24" s="14">
+        <v>12</v>
+      </c>
+      <c r="M24" s="14">
+        <v>428</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>100</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
       <c r="T24" s="14"/>
       <c r="U24" s="14"/>
-      <c r="V24" s="14"/>
+      <c r="V24" s="14">
+        <v>1</v>
+      </c>
       <c r="W24" s="14"/>
       <c r="X24" s="14"/>
       <c r="Y24" s="15"/>
@@ -20144,23 +20203,37 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>0</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>1</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>2</v>
+      </c>
+      <c r="L31" s="23">
+        <v>0</v>
+      </c>
+      <c r="M31" s="23">
+        <v>43</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>100</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
       <c r="T31" s="23"/>
       <c r="U31" s="23"/>
-      <c r="V31" s="23"/>
+      <c r="V31" s="23">
+        <v>1</v>
+      </c>
       <c r="W31" s="23"/>
       <c r="X31" s="61"/>
       <c r="Y31" s="24"/>
@@ -20172,23 +20245,37 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>3</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>28</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>67</v>
+      </c>
+      <c r="L32" s="28">
+        <v>12</v>
+      </c>
+      <c r="M32" s="28">
+        <v>385</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
       <c r="T32" s="28"/>
       <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
+      <c r="V32" s="28">
+        <v>0</v>
+      </c>
       <c r="W32" s="28"/>
       <c r="X32" s="63"/>
       <c r="Y32" s="29"/>
@@ -20220,47 +20307,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -20310,38 +20397,50 @@
       <c r="S35" s="70"/>
       <c r="T35" s="70"/>
       <c r="U35" s="71"/>
-      <c r="V35" s="82"/>
-      <c r="W35" s="82"/>
-      <c r="X35" s="82"/>
-      <c r="Y35" s="82"/>
+      <c r="V35" s="84"/>
+      <c r="W35" s="84"/>
+      <c r="X35" s="84"/>
+      <c r="Y35" s="84"/>
     </row>
     <row r="36" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="46">
+        <v>3</v>
+      </c>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
+      <c r="F36" s="42">
+        <v>457</v>
+      </c>
       <c r="G36" s="42"/>
       <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
+      <c r="I36" s="42">
+        <v>4</v>
+      </c>
       <c r="J36" s="42"/>
       <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
+      <c r="L36" s="42">
+        <v>67</v>
+      </c>
       <c r="M36" s="42"/>
       <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
-      <c r="P36" s="42"/>
+      <c r="O36" s="42">
+        <v>11</v>
+      </c>
+      <c r="P36" s="42">
+        <v>6</v>
+      </c>
       <c r="Q36" s="43"/>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
-      <c r="U36" s="82"/>
-      <c r="V36" s="82"/>
-      <c r="W36" s="82"/>
-      <c r="X36" s="82"/>
-      <c r="Y36" s="82"/>
+      <c r="U36" s="84"/>
+      <c r="V36" s="84"/>
+      <c r="W36" s="84"/>
+      <c r="X36" s="84"/>
+      <c r="Y36" s="84"/>
     </row>
     <row r="37" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="53"/>
@@ -20363,11 +20462,11 @@
       <c r="R37" s="72"/>
       <c r="S37" s="44"/>
       <c r="T37" s="44"/>
-      <c r="U37" s="82"/>
-      <c r="V37" s="82"/>
-      <c r="W37" s="82"/>
-      <c r="X37" s="82"/>
-      <c r="Y37" s="82"/>
+      <c r="U37" s="84"/>
+      <c r="V37" s="84"/>
+      <c r="W37" s="84"/>
+      <c r="X37" s="84"/>
+      <c r="Y37" s="84"/>
     </row>
     <row r="38" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="53"/>
@@ -20389,11 +20488,11 @@
       <c r="R38" s="72"/>
       <c r="S38" s="44"/>
       <c r="T38" s="44"/>
-      <c r="U38" s="82"/>
-      <c r="V38" s="82"/>
-      <c r="W38" s="82"/>
-      <c r="X38" s="82"/>
-      <c r="Y38" s="82"/>
+      <c r="U38" s="84"/>
+      <c r="V38" s="84"/>
+      <c r="W38" s="84"/>
+      <c r="X38" s="84"/>
+      <c r="Y38" s="84"/>
     </row>
     <row r="39" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="53"/>
@@ -20415,11 +20514,11 @@
       <c r="R39" s="72"/>
       <c r="S39" s="44"/>
       <c r="T39" s="44"/>
-      <c r="U39" s="82"/>
-      <c r="V39" s="82"/>
-      <c r="W39" s="82"/>
-      <c r="X39" s="82"/>
-      <c r="Y39" s="82"/>
+      <c r="U39" s="84"/>
+      <c r="V39" s="84"/>
+      <c r="W39" s="84"/>
+      <c r="X39" s="84"/>
+      <c r="Y39" s="84"/>
     </row>
     <row r="40" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="53"/>
@@ -20441,11 +20540,11 @@
       <c r="R40" s="72"/>
       <c r="S40" s="44"/>
       <c r="T40" s="44"/>
-      <c r="U40" s="82"/>
-      <c r="V40" s="82"/>
-      <c r="W40" s="82"/>
-      <c r="X40" s="82"/>
-      <c r="Y40" s="82"/>
+      <c r="U40" s="84"/>
+      <c r="V40" s="84"/>
+      <c r="W40" s="84"/>
+      <c r="X40" s="84"/>
+      <c r="Y40" s="84"/>
     </row>
     <row r="41" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="54"/>
@@ -20468,36 +20567,48 @@
       <c r="S41" s="74"/>
       <c r="T41" s="74"/>
       <c r="U41" s="75"/>
-      <c r="V41" s="82"/>
-      <c r="W41" s="82"/>
-      <c r="X41" s="82"/>
-      <c r="Y41" s="82"/>
+      <c r="V41" s="84"/>
+      <c r="W41" s="84"/>
+      <c r="X41" s="84"/>
+      <c r="Y41" s="84"/>
     </row>
     <row r="42" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="46"/>
+      <c r="C42" s="46">
+        <v>3</v>
+      </c>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
+      <c r="F42" s="42">
+        <v>457</v>
+      </c>
       <c r="G42" s="42"/>
       <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
+      <c r="I42" s="42">
+        <v>4</v>
+      </c>
       <c r="J42" s="42"/>
       <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
+      <c r="L42" s="42">
+        <v>67</v>
+      </c>
       <c r="M42" s="42"/>
       <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
+      <c r="O42" s="42">
+        <v>11</v>
+      </c>
+      <c r="P42" s="42">
+        <v>6</v>
+      </c>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -20533,17 +20644,21 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96">
+        <v>506</v>
+      </c>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96">
+        <v>12</v>
+      </c>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -20903,12 +21018,18 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="13">
+        <v>2</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>78</v>
+      </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>97</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -20923,7 +21044,9 @@
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
+      <c r="W8" s="14">
+        <v>1</v>
+      </c>
       <c r="X8" s="59"/>
       <c r="Y8" s="15"/>
     </row>
@@ -21091,12 +21214,18 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>78</v>
+      </c>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>96</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -21111,7 +21240,9 @@
       <c r="T15" s="23"/>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
+      <c r="W15" s="23">
+        <v>0</v>
+      </c>
       <c r="X15" s="61"/>
       <c r="Y15" s="24"/>
     </row>
@@ -21119,12 +21250,18 @@
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
+      <c r="C16" s="57">
+        <v>1</v>
+      </c>
+      <c r="D16" s="58">
+        <v>0</v>
+      </c>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>95</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -21139,7 +21276,9 @@
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
+      <c r="W16" s="56">
+        <v>1</v>
+      </c>
       <c r="X16" s="62"/>
       <c r="Y16" s="29"/>
     </row>
@@ -21505,17 +21644,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>3</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>3</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>20</v>
+      </c>
+      <c r="L24" s="14">
+        <v>12</v>
+      </c>
+      <c r="M24" s="14">
+        <v>455</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14">
+        <v>16</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -21691,17 +21842,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>0</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>3</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>0</v>
+      </c>
+      <c r="L31" s="23">
+        <v>0</v>
+      </c>
+      <c r="M31" s="23">
+        <v>88</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23">
+        <v>16</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -21719,17 +21882,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>3</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>0</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>20</v>
+      </c>
+      <c r="L32" s="28">
+        <v>12</v>
+      </c>
+      <c r="M32" s="28">
+        <v>367</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -21767,47 +21942,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -21866,21 +22041,43 @@
       <c r="B36" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="46">
+        <v>5</v>
+      </c>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
+      <c r="F36" s="42">
+        <v>378</v>
+      </c>
+      <c r="G36" s="42">
+        <v>6</v>
+      </c>
       <c r="H36" s="42"/>
       <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
-      <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="J36" s="42">
+        <v>1</v>
+      </c>
+      <c r="K36" s="42">
+        <v>9</v>
+      </c>
+      <c r="L36" s="42">
+        <v>13</v>
+      </c>
+      <c r="M36" s="42">
+        <v>7</v>
+      </c>
+      <c r="N36" s="42">
+        <v>2</v>
+      </c>
+      <c r="O36" s="42">
+        <v>2</v>
+      </c>
+      <c r="P36" s="42">
+        <v>6</v>
+      </c>
+      <c r="Q36" s="43">
+        <v>8</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -22024,27 +22221,49 @@
       <c r="B42" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="46"/>
+      <c r="C42" s="46">
+        <v>5</v>
+      </c>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
+      <c r="F42" s="42">
+        <v>378</v>
+      </c>
+      <c r="G42" s="42">
+        <v>6</v>
+      </c>
       <c r="H42" s="42"/>
       <c r="I42" s="42"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="J42" s="42">
+        <v>1</v>
+      </c>
+      <c r="K42" s="42">
+        <v>9</v>
+      </c>
+      <c r="L42" s="42">
+        <v>13</v>
+      </c>
+      <c r="M42" s="42">
+        <v>7</v>
+      </c>
+      <c r="N42" s="42">
+        <v>2</v>
+      </c>
+      <c r="O42" s="42">
+        <v>2</v>
+      </c>
+      <c r="P42" s="42">
+        <v>6</v>
+      </c>
+      <c r="Q42" s="43">
+        <v>8</v>
+      </c>
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -22080,17 +22299,22 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96">
+        <f>1+11+1+3+20+12+367</f>
+        <v>415</v>
+      </c>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96">
+        <v>5</v>
+      </c>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -23311,47 +23535,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -23583,12 +23807,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -24842,47 +25066,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -25114,12 +25338,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -25155,17 +25379,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -26389,47 +26613,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -26661,12 +26885,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -26702,17 +26926,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -27936,47 +28160,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -28208,12 +28432,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -28249,17 +28473,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -29480,47 +29704,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -29752,12 +29976,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -31011,47 +31235,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -31283,12 +31507,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -31324,17 +31548,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -32558,47 +32782,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -32830,12 +33054,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -32871,17 +33095,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -34105,47 +34329,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -34377,12 +34601,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -34418,17 +34642,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -35654,47 +35878,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -35926,12 +36150,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -35967,17 +36191,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -37198,47 +37422,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -37470,12 +37694,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -38729,47 +38953,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -39001,12 +39225,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -39042,17 +39266,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -40276,47 +40500,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -40548,12 +40772,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -40589,17 +40813,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -41823,47 +42047,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -42095,12 +42319,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -42136,17 +42360,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -43370,47 +43594,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -43642,12 +43866,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -43683,17 +43907,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -44917,47 +45141,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -45189,12 +45413,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -45230,17 +45454,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="96"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="C45" s="96"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -46461,47 +46685,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -46733,12 +46957,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -48046,47 +48270,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -48362,12 +48586,12 @@
       <c r="Q42" s="43">
         <v>13</v>
       </c>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -48403,23 +48627,23 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>1+2+1+32+9+283</f>
         <v>328</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95">
+      <c r="C45" s="96">
         <f>8</f>
         <v>8</v>
       </c>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -49733,47 +49957,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -50045,12 +50269,12 @@
       <c r="Q42" s="43">
         <v>4</v>
       </c>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -50086,23 +50310,23 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>1+1+25+1+2+168+1+6+487+2+1</f>
         <v>695</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95">
+      <c r="C45" s="96">
         <f>8</f>
         <v>8</v>
       </c>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -51398,47 +51622,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="91"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="93" t="s">
+      <c r="D34" s="92"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="91"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="93" t="s">
+      <c r="G34" s="92"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="91"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="93" t="s">
+      <c r="J34" s="92"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="91"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="94" t="s">
+      <c r="M34" s="92"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="94"/>
-      <c r="Q34" s="94"/>
-      <c r="R34" s="84" t="s">
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="85"/>
-      <c r="T34" s="85"/>
-      <c r="U34" s="86"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="87"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="90"/>
+      <c r="B35" s="91"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -51710,12 +51934,12 @@
       <c r="Q42" s="43">
         <v>15</v>
       </c>
-      <c r="R42" s="87" t="s">
+      <c r="R42" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="88"/>
-      <c r="T42" s="88"/>
-      <c r="U42" s="88"/>
+      <c r="S42" s="89"/>
+      <c r="T42" s="89"/>
+      <c r="U42" s="89"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -51751,23 +51975,23 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="95">
+      <c r="C44" s="96">
         <f>17+2+1+2+81+14+428</f>
         <v>545</v>
       </c>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="96"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="95">
+      <c r="C45" s="96">
         <f>3</f>
         <v>3</v>
       </c>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
+      <c r="D45" s="96"/>
+      <c r="E45" s="96"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>